<commit_message>
Automatically updating raw market quote data
</commit_message>
<xml_diff>
--- a/data_raw/CME_BRR_latest.xlsx
+++ b/data_raw/CME_BRR_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D837"/>
+  <dimension ref="A1:D841"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13826,6 +13826,70 @@
         <v>82480.33</v>
       </c>
     </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B838" t="n">
+        <v>82834.44</v>
+      </c>
+      <c r="C838" t="n">
+        <v>82976.42</v>
+      </c>
+      <c r="D838" t="n">
+        <v>82637.10000000001</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B839" t="n">
+        <v>83022.35000000001</v>
+      </c>
+      <c r="C839" t="n">
+        <v>83623.48</v>
+      </c>
+      <c r="D839" t="n">
+        <v>83003.17</v>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B840" t="n">
+        <v>82721.17</v>
+      </c>
+      <c r="C840" t="n">
+        <v>82528.45</v>
+      </c>
+      <c r="D840" t="n">
+        <v>84010.35000000001</v>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B841" t="n">
+        <v>83524.64999999999</v>
+      </c>
+      <c r="C841" t="n">
+        <v>83140.61</v>
+      </c>
+      <c r="D841" t="n">
+        <v>83733.36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>